<commit_message>
Updated app file names
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saichunduru\fifa wc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9E4764-16D8-4B41-BB1F-8273E325FDAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0532C8DB-D847-471A-8A20-724D72C77760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="17460" windowHeight="10260" xr2:uid="{E67833B8-4FEA-401B-A1B4-AB5D5161C38E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="52">
   <si>
     <t>Pot A</t>
   </si>
@@ -159,6 +159,42 @@
   </si>
   <si>
     <t>Spain</t>
+  </si>
+  <si>
+    <t>The Craw</t>
+  </si>
+  <si>
+    <t>Pique Blinders</t>
+  </si>
+  <si>
+    <t>Angus</t>
+  </si>
+  <si>
+    <t>England</t>
+  </si>
+  <si>
+    <t>Curaçao</t>
+  </si>
+  <si>
+    <t>It's Coming Home</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Gwinyeo</t>
+  </si>
+  <si>
+    <t>GemmaMorgan</t>
+  </si>
+  <si>
+    <t>DRedmond</t>
+  </si>
+  <si>
+    <t>Scorerg</t>
+  </si>
+  <si>
+    <t>Egypt</t>
   </si>
 </sst>
 </file>
@@ -537,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1271A6DF-7B4F-4F21-A272-DFA4D7BFB8B4}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="21.04296875" customWidth="1"/>
@@ -768,6 +804,142 @@
         <v>28</v>
       </c>
     </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.75">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
App and users updated
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saichunduru\fifa wc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C4475E-8363-4F6F-A9EA-045A311E51BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1830E0B-213B-47FB-889C-DBE43DCAF4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="17460" windowHeight="10260" xr2:uid="{E67833B8-4FEA-401B-A1B4-AB5D5161C38E}"/>
+    <workbookView xWindow="2135" yWindow="2135" windowWidth="12960" windowHeight="7290" xr2:uid="{E67833B8-4FEA-401B-A1B4-AB5D5161C38E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="83">
   <si>
     <t>Pot A</t>
   </si>
@@ -273,6 +273,21 @@
   </si>
   <si>
     <t>It's Coming Home1</t>
+  </si>
+  <si>
+    <t>Lavina</t>
+  </si>
+  <si>
+    <t>Uruguay</t>
+  </si>
+  <si>
+    <t>Qatar</t>
+  </si>
+  <si>
+    <t>Lukas</t>
+  </si>
+  <si>
+    <t>Canada</t>
   </si>
 </sst>
 </file>
@@ -651,7 +666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1271A6DF-7B4F-4F21-A272-DFA4D7BFB8B4}">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="21.04296875" customWidth="1"/>
@@ -1307,6 +1322,40 @@
         <v>14</v>
       </c>
     </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C39" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" t="s">
+        <v>80</v>
+      </c>
+      <c r="E39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A40" t="s">
+        <v>81</v>
+      </c>
+      <c r="B40" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" t="s">
+        <v>37</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>